<commit_message>
update drive-away dolls watched
</commit_message>
<xml_diff>
--- a/content/database.xlsx
+++ b/content/database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hannah\life\dabad2_0\dabad\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFC7E6E3-2575-4CBA-BFDA-7E34008DE727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A7FC1D-89CB-4026-9D46-A49B7858A3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{730DD696-8E95-48A8-8025-F5D06081233D}"/>
   </bookViews>
@@ -16279,7 +16279,7 @@
         <v>763</v>
       </c>
       <c r="G135" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H135" s="4"/>
       <c r="I135" s="6" t="s">

</xml_diff>